<commit_message>
feat(account-review): add Source of Funds check (R-SOF-CHECK) case
Adds a 7th account-review case: a source-of-funds-check skill runs all
four gates (documents, wealth ratio, screening, dealing calendar) in
full regardless of outcome, escalating to Compliance only on a gate
failure and confirming with no email when all four pass.

- contract: add case_action.sof_transaction_amount / sof_folder_id
- server.py + import_plan.py: map the two new fields end to end
- cases.json: sof-check entry, skip_default_email_note for the
  conditional (pass = no email) ending
- CaseActionBar.astro: make the generic "always call send_email"
  trailing sentence conditional on skip_default_email_note
- docs/07-sof-check.md: matching diagram for the new case, wired into
  the docs index and 06's nav
</commit_message>
<xml_diff>
--- a/tutorials/mcp/mcp_dashboards/datasets/account_review/fastmcp/data/account_review_dataset.xlsx
+++ b/tutorials/mcp/mcp_dashboards/datasets/account_review/fastmcp/data/account_review_dataset.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CS17"/>
+  <dimension ref="A1:CU17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1084,6 +1084,16 @@
           <t>Suitability Outcome</t>
         </is>
       </c>
+      <c r="CT4" t="inlineStr">
+        <is>
+          <t>Sof Transaction Amount</t>
+        </is>
+      </c>
+      <c r="CU4" t="inlineStr">
+        <is>
+          <t>Sof Folder Id</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -5820,7 +5830,239 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CH-priv-0472</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Thomas Bürki</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Private Wealth</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Swiss</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>32000000</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Incoming USD 3,000,000 subscription flagged for mandatory Source of Funds review.</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>R-SOF-CHECK</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Run Source of Funds check</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Client DB</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>2020-05-14</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>passport, proof_of_address</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>1975-02-10</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Managing partner, private holding</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>12 Bahnhofstrasse, 8001 Zürich, Switzerland</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>t.buerki@example.ch</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>+41 79 555 0472</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Married</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>CRD-CH-0472</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>Run Source of Funds check</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>Incoming USD 3,000,000 subscription flagged for mandatory Source of Funds review before allotment.</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>Run SoF check</t>
+        </is>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>Advisory — Balanced</t>
+        </is>
+      </c>
+      <c r="BZ17" t="inlineStr">
+        <is>
+          <t>Professional — MiFID elective</t>
+        </is>
+      </c>
+      <c r="CA17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB17" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CO17" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP17" t="inlineStr">
+        <is>
+          <t>5+ years</t>
+        </is>
+      </c>
+      <c r="CQ17" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="CR17" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="CS17" t="inlineStr">
+        <is>
+          <t>Aligned with Balanced mandate</t>
+        </is>
+      </c>
+      <c r="CT17" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="CU17" t="inlineStr">
+        <is>
+          <t>scope_zmwtzb2r9e6rwixcrx65md6n</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:Z16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update with new use cases
</commit_message>
<xml_diff>
--- a/tutorials/mcp/mcp_dashboards/datasets/account_review/fastmcp/data/account_review_dataset.xlsx
+++ b/tutorials/mcp/mcp_dashboards/datasets/account_review/fastmcp/data/account_review_dataset.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CU17"/>
+  <dimension ref="A1:CU18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1084,12 +1084,12 @@
           <t>Suitability Outcome</t>
         </is>
       </c>
-      <c r="CT4" t="inlineStr">
+      <c r="CT4" s="3" t="inlineStr">
         <is>
           <t>Sof Transaction Amount</t>
         </is>
       </c>
-      <c r="CU4" t="inlineStr">
+      <c r="CU4" s="3" t="inlineStr">
         <is>
           <t>Sof Folder Id</t>
         </is>
@@ -5831,75 +5831,76 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>CH-priv-0472</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Thomas Bürki</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Private Wealth</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Balanced</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Swiss</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="5" t="n">
         <v>32000000</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>Review required</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Incoming USD 3,000,000 subscription flagged for mandatory Source of Funds review.</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>R-SOF-CHECK</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Run Source of Funds check</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -5909,47 +5910,48 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="T17" s="4" t="inlineStr">
         <is>
           <t>2027-06-01</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="U17" s="4" t="inlineStr">
         <is>
           <t>2027-06-01</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="V17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="W17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="X17" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Y17" s="4" t="inlineStr">
         <is>
           <t>Client DB</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="Z17" s="4" t="inlineStr">
         <is>
           <t>2020-05-14</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AA17" s="4" t="inlineStr">
         <is>
           <t>passport, proof_of_address</t>
         </is>
@@ -6059,7 +6061,242 @@
       </c>
       <c r="CU17" t="inlineStr">
         <is>
-          <t>scope_zmwtzb2r9e6rwixcrx65md6n</t>
+          <t>scope_eyz8sc3ijxex2nj4mv22oo9p</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CH-priv-0473</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Thomas Bürki</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Private Wealth</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Swiss</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>32000000</v>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>Review required</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Incoming USD 3,000,000 subscription flagged for mandatory Source of Funds review.</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>R-SOF-CHECK</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>Run Source of Funds check</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>Client DB</t>
+        </is>
+      </c>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>2020-05-14</t>
+        </is>
+      </c>
+      <c r="AA18" s="4" t="inlineStr">
+        <is>
+          <t>passport, proof_of_address</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>1975-02-10</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Managing partner, private holding</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>12 Bahnhofstrasse, 8001 Zürich, Switzerland</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>t.buerki@example.ch</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>+41 79 555 0472</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>Married</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>CRD-CH-0473</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>Run Source of Funds check</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>Incoming USD 3,000,000 subscription flagged for mandatory Source of Funds review before allotment.</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>Run SoF check</t>
+        </is>
+      </c>
+      <c r="BM18" t="inlineStr">
+        <is>
+          <t>Advisory — Balanced</t>
+        </is>
+      </c>
+      <c r="BZ18" t="inlineStr">
+        <is>
+          <t>Professional — MiFID elective</t>
+        </is>
+      </c>
+      <c r="CA18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB18" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CO18" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP18" t="inlineStr">
+        <is>
+          <t>5+ years</t>
+        </is>
+      </c>
+      <c r="CQ18" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="CR18" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="CS18" t="inlineStr">
+        <is>
+          <t>Aligned with Balanced mandate</t>
+        </is>
+      </c>
+      <c r="CT18" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="CU18" t="inlineStr">
+        <is>
+          <t>scope_qblw3b640c9xm8n4cqhggfdu</t>
         </is>
       </c>
     </row>

</xml_diff>